<commit_message>
Tighten module audit classification baseline
</commit_message>
<xml_diff>
--- a/reports/module-data-integration-audit/2026-07-27/CONSUMPTION_PROJECTION_MATRIX.xlsx
+++ b/reports/module-data-integration-audit/2026-07-27/CONSUMPTION_PROJECTION_MATRIX.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumption" sheetId="1" r:id="Reca9d13301254b4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumption" sheetId="1" r:id="R94c0c2f8efd24761"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -345,10 +345,10 @@
         <x:v>Tower</x:v>
       </x:c>
       <x:c r="B2" s="5" t="str">
-        <x:v>cio_tower.mart_ai_portfolio</x:v>
+        <x:v>cio_tower.facts</x:v>
       </x:c>
       <x:c r="C2" s="5" t="str">
-        <x:v>existing derived read model</x:v>
+        <x:v>candidate shared projection</x:v>
       </x:c>
       <x:c r="D2" s="5" t="str">
         <x:v>Cube; Nexus; aVa; Superset; Observable; module dashboards</x:v>
@@ -368,7 +368,7 @@
         <x:v>Tower</x:v>
       </x:c>
       <x:c r="B3" s="5" t="str">
-        <x:v>cio_tower.mart_command_center</x:v>
+        <x:v>cio_tower.mart_ai_portfolio</x:v>
       </x:c>
       <x:c r="C3" s="5" t="str">
         <x:v>existing derived read model</x:v>
@@ -391,7 +391,7 @@
         <x:v>Tower</x:v>
       </x:c>
       <x:c r="B4" s="5" t="str">
-        <x:v>cio_tower.mart_cxo_actions</x:v>
+        <x:v>cio_tower.mart_command_center</x:v>
       </x:c>
       <x:c r="C4" s="5" t="str">
         <x:v>existing derived read model</x:v>
@@ -414,7 +414,7 @@
         <x:v>Tower</x:v>
       </x:c>
       <x:c r="B5" s="5" t="str">
-        <x:v>cio_tower.mart_evidence_lineage</x:v>
+        <x:v>cio_tower.mart_cxo_actions</x:v>
       </x:c>
       <x:c r="C5" s="5" t="str">
         <x:v>existing derived read model</x:v>
@@ -437,7 +437,7 @@
         <x:v>Tower</x:v>
       </x:c>
       <x:c r="B6" s="5" t="str">
-        <x:v>cio_tower.mart_program_decision_lanes</x:v>
+        <x:v>cio_tower.mart_evidence_lineage</x:v>
       </x:c>
       <x:c r="C6" s="5" t="str">
         <x:v>existing derived read model</x:v>
@@ -460,7 +460,7 @@
         <x:v>Tower</x:v>
       </x:c>
       <x:c r="B7" s="5" t="str">
-        <x:v>cio_tower.mart_required_field_gaps</x:v>
+        <x:v>cio_tower.mart_program_decision_lanes</x:v>
       </x:c>
       <x:c r="C7" s="5" t="str">
         <x:v>existing derived read model</x:v>
@@ -483,7 +483,7 @@
         <x:v>Tower</x:v>
       </x:c>
       <x:c r="B8" s="5" t="str">
-        <x:v>cio_tower.mart_value_funnel</x:v>
+        <x:v>cio_tower.mart_required_field_gaps</x:v>
       </x:c>
       <x:c r="C8" s="5" t="str">
         <x:v>existing derived read model</x:v>
@@ -506,7 +506,7 @@
         <x:v>Tower</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>public.ai_control_tower_lens_mv</x:v>
+        <x:v>cio_tower.mart_value_funnel</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str">
         <x:v>existing derived read model</x:v>
@@ -529,10 +529,10 @@
         <x:v>Tower</x:v>
       </x:c>
       <x:c r="B10" s="5" t="str">
-        <x:v>public.mart</x:v>
+        <x:v>cio_tower.measure_results</x:v>
       </x:c>
       <x:c r="C10" s="5" t="str">
-        <x:v>existing derived read model</x:v>
+        <x:v>candidate shared projection</x:v>
       </x:c>
       <x:c r="D10" s="5" t="str">
         <x:v>Cube; Nexus; aVa; Superset; Observable; module dashboards</x:v>
@@ -552,7 +552,7 @@
         <x:v>Tower</x:v>
       </x:c>
       <x:c r="B11" s="5" t="str">
-        <x:v>public.MART</x:v>
+        <x:v>public.ai_control_atlas_context_packs</x:v>
       </x:c>
       <x:c r="C11" s="5" t="str">
         <x:v>candidate shared projection</x:v>
@@ -571,25 +571,140 @@
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
-      <x:c r="A12" s="6" t="str">
-        <x:v>Tower</x:v>
-      </x:c>
-      <x:c r="B12" s="6" t="str">
+      <x:c r="A12" s="5" t="str">
+        <x:v>Tower</x:v>
+      </x:c>
+      <x:c r="B12" s="5" t="str">
+        <x:v>public.ai_control_tower_lens_mv</x:v>
+      </x:c>
+      <x:c r="C12" s="5" t="str">
+        <x:v>existing derived read model</x:v>
+      </x:c>
+      <x:c r="D12" s="5" t="str">
+        <x:v>Cube; Nexus; aVa; Superset; Observable; module dashboards</x:v>
+      </x:c>
+      <x:c r="E12" s="5" t="str">
+        <x:v>Domain publication/outbox to stable consumption projection</x:v>
+      </x:c>
+      <x:c r="F12" s="5" t="str">
+        <x:v>Compare existing module output to projection output before switching consumers</x:v>
+      </x:c>
+      <x:c r="G12" s="5" t="str">
+        <x:v>Keep domain read path until projection parity and signed-in proof pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="5" t="str">
+        <x:v>Tower</x:v>
+      </x:c>
+      <x:c r="B13" s="5" t="str">
         <x:v>public.tower_budget_rollups</x:v>
       </x:c>
-      <x:c r="C12" s="6" t="str">
+      <x:c r="C13" s="5" t="str">
         <x:v>candidate shared projection</x:v>
       </x:c>
-      <x:c r="D12" s="6" t="str">
-        <x:v>Cube; Nexus; aVa; Superset; Observable; module dashboards</x:v>
-      </x:c>
-      <x:c r="E12" s="6" t="str">
-        <x:v>Domain publication/outbox to stable consumption projection</x:v>
-      </x:c>
-      <x:c r="F12" s="6" t="str">
-        <x:v>Compare existing module output to projection output before switching consumers</x:v>
-      </x:c>
-      <x:c r="G12" s="6" t="str">
+      <x:c r="D13" s="5" t="str">
+        <x:v>Cube; Nexus; aVa; Superset; Observable; module dashboards</x:v>
+      </x:c>
+      <x:c r="E13" s="5" t="str">
+        <x:v>Domain publication/outbox to stable consumption projection</x:v>
+      </x:c>
+      <x:c r="F13" s="5" t="str">
+        <x:v>Compare existing module output to projection output before switching consumers</x:v>
+      </x:c>
+      <x:c r="G13" s="5" t="str">
+        <x:v>Keep domain read path until projection parity and signed-in proof pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="5" t="str">
+        <x:v>Tower</x:v>
+      </x:c>
+      <x:c r="B14" s="5" t="str">
+        <x:v>public.tower_cmdb_dependencies</x:v>
+      </x:c>
+      <x:c r="C14" s="5" t="str">
+        <x:v>candidate shared projection</x:v>
+      </x:c>
+      <x:c r="D14" s="5" t="str">
+        <x:v>Cube; Nexus; aVa; Superset; Observable; module dashboards</x:v>
+      </x:c>
+      <x:c r="E14" s="5" t="str">
+        <x:v>Domain publication/outbox to stable consumption projection</x:v>
+      </x:c>
+      <x:c r="F14" s="5" t="str">
+        <x:v>Compare existing module output to projection output before switching consumers</x:v>
+      </x:c>
+      <x:c r="G14" s="5" t="str">
+        <x:v>Keep domain read path until projection parity and signed-in proof pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="5" t="str">
+        <x:v>Tower</x:v>
+      </x:c>
+      <x:c r="B15" s="5" t="str">
+        <x:v>public.tower_dora_metrics</x:v>
+      </x:c>
+      <x:c r="C15" s="5" t="str">
+        <x:v>candidate shared projection</x:v>
+      </x:c>
+      <x:c r="D15" s="5" t="str">
+        <x:v>Cube; Nexus; aVa; Superset; Observable; module dashboards</x:v>
+      </x:c>
+      <x:c r="E15" s="5" t="str">
+        <x:v>Domain publication/outbox to stable consumption projection</x:v>
+      </x:c>
+      <x:c r="F15" s="5" t="str">
+        <x:v>Compare existing module output to projection output before switching consumers</x:v>
+      </x:c>
+      <x:c r="G15" s="5" t="str">
+        <x:v>Keep domain read path until projection parity and signed-in proof pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="5" t="str">
+        <x:v>Tower</x:v>
+      </x:c>
+      <x:c r="B16" s="5" t="str">
+        <x:v>public.tower_program_financials</x:v>
+      </x:c>
+      <x:c r="C16" s="5" t="str">
+        <x:v>candidate shared projection</x:v>
+      </x:c>
+      <x:c r="D16" s="5" t="str">
+        <x:v>Cube; Nexus; aVa; Superset; Observable; module dashboards</x:v>
+      </x:c>
+      <x:c r="E16" s="5" t="str">
+        <x:v>Domain publication/outbox to stable consumption projection</x:v>
+      </x:c>
+      <x:c r="F16" s="5" t="str">
+        <x:v>Compare existing module output to projection output before switching consumers</x:v>
+      </x:c>
+      <x:c r="G16" s="5" t="str">
+        <x:v>Keep domain read path until projection parity and signed-in proof pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="6" t="str">
+        <x:v>Tower</x:v>
+      </x:c>
+      <x:c r="B17" s="6" t="str">
+        <x:v>public.tower_vendor_spend</x:v>
+      </x:c>
+      <x:c r="C17" s="6" t="str">
+        <x:v>candidate shared projection</x:v>
+      </x:c>
+      <x:c r="D17" s="6" t="str">
+        <x:v>Cube; Nexus; aVa; Superset; Observable; module dashboards</x:v>
+      </x:c>
+      <x:c r="E17" s="6" t="str">
+        <x:v>Domain publication/outbox to stable consumption projection</x:v>
+      </x:c>
+      <x:c r="F17" s="6" t="str">
+        <x:v>Compare existing module output to projection output before switching consumers</x:v>
+      </x:c>
+      <x:c r="G17" s="6" t="str">
         <x:v>Keep domain read path until projection parity and signed-in proof pass</x:v>
       </x:c>
     </x:row>

</xml_diff>